<commit_message>
Small shunt scaling change and validation tweaks.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/CSTARS.xlsx
+++ b/data/human/adult/validation/Scenarios/CSTARS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B08C5B4-4D05-4BB3-8C48-745C58EF3914}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79A12A9F-0610-4DEF-B683-7650FB4E905C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27180" yWindow="5040" windowWidth="27555" windowHeight="24945" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28410" yWindow="4725" windowWidth="27555" windowHeight="24945" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1569" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1569" uniqueCount="206">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -865,34 +865,6 @@
     <t>musch2008relation</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 27, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.25, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 16, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 27, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.25, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 16, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } }
-  }}
-}</t>
-  </si>
-  <si>
     <t>Learning Objectives:
  - Recognize mild ARDS
  - Recognize hypventilation (rate too low and patient not triggering additional breaths)
@@ -910,15 +882,7 @@
 </t>
   </si>
   <si>
-    <t>Increase FiO2.  Patient transport has ended.
-Recommended Actions:
- - Consider PC-CMV to liberate inspiratory volume and flow
- - Monitor for excessive tidal volume
-Ventilator settings are updated to:
- - FiO2: 0.4 -&gt; 0.5
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.567    | NA          | 27           | NA  | 1.25    | 16      | 10            | 0.5 |</t>
+    <t>{ "AdvanceTime": { "Time": { "ScalarTime": { "Value": 1, "Unit": "min" }}}}</t>
   </si>
   <si>
     <t>Increase PEEP.
@@ -929,10 +893,64 @@
  - PEEP: 5 -&gt; 10 cmH2O
 | Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.567    | NA          | 27           | NA  | 1.25    | 16      | 10            | 0.4 |</t>
+| VC-CMV | 0.567    | NA          | 27           | NA  | 1.25    | 16      | 15            | 0.4 |</t>
   </si>
   <si>
-    <t>{ "AdvanceTime": { "Time": { "ScalarTime": { "Value": 1, "Unit": "min" }}}}</t>
+    <t>Increase FiO2.  Patient transport has ended.
+Recommended Actions:
+ - Consider PC-CMV to liberate inspiratory volume and flow
+ - Monitor for excessive tidal volume
+Ventilator settings are updated to:
+ - FiO2: 0.4 -&gt; 0.5
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.567    | NA          | 27           | NA  | 1.25    | 16      | 15            | 0.5 |</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 27, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.25, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 15, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 16, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 27, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 1.25, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 15, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 16, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "PatientAction": { "AcuteRespiratoryDistressSyndromeExacerbation":
+  {
+    "Severity": [ 
+      { "Compartment": "LeftLung", "Severity": { "Scalar0To1": { "Value": 0.27 }}},
+      { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.27 }}}]
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "PatientAction": { "AcuteRespiratoryDistressSyndromeExacerbation":
+  {
+    "Severity": [ 
+      { "Compartment": "LeftLung", "Severity": { "Scalar0To1": { "Value": 0.57 }}},
+      { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.57 }}}]
+  }}
+}</t>
   </si>
 </sst>
 </file>
@@ -1730,14 +1748,14 @@
         <v>1</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>153</v>
+        <v>204</v>
       </c>
       <c r="C12" s="19"/>
       <c r="D12" s="19"/>
       <c r="E12" s="19"/>
       <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -2034,14 +2052,14 @@
         <v>2</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>154</v>
+        <v>205</v>
       </c>
       <c r="C27" s="19"/>
       <c r="D27" s="19"/>
       <c r="E27" s="19"/>
       <c r="F27" s="19"/>
       <c r="G27" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H27" s="9"/>
     </row>
@@ -2324,14 +2342,14 @@
         <v>3</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C40" s="26"/>
       <c r="D40" s="26"/>
       <c r="E40" s="26"/>
       <c r="F40" s="27"/>
       <c r="G40" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="H40" s="10"/>
     </row>
@@ -2542,7 +2560,7 @@
         <v>4</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C50" s="26"/>
       <c r="D50" s="26"/>
@@ -2970,7 +2988,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -3346,7 +3364,7 @@
         <v>2</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C33" s="19"/>
       <c r="D33" s="19"/>
@@ -3708,7 +3726,7 @@
         <v>3</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C49" s="19"/>
       <c r="D49" s="19"/>
@@ -4331,7 +4349,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -9741,7 +9759,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
@@ -24281,7 +24299,7 @@
         <v>3</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C45" s="19"/>
       <c r="D45" s="19"/>
@@ -31848,7 +31866,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -32116,7 +32134,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C28" s="19"/>
       <c r="D28" s="19"/>
@@ -32360,7 +32378,7 @@
         <v>3</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C39" s="19"/>
       <c r="D39" s="19"/>
@@ -32816,7 +32834,7 @@
         <v>1</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -33108,7 +33126,7 @@
         <v>2</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C29" s="19"/>
       <c r="D29" s="19"/>
@@ -33376,7 +33394,7 @@
         <v>3</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C41" s="19"/>
       <c r="D41" s="19"/>
@@ -33744,7 +33762,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
@@ -34084,7 +34102,7 @@
         <v>2</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C30" s="19"/>
       <c r="D30" s="19"/>
@@ -34352,7 +34370,7 @@
         <v>3</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C42" s="19"/>
       <c r="D42" s="19"/>
@@ -34719,7 +34737,7 @@
         <v>1</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C15" s="19"/>
       <c r="D15" s="19"/>
@@ -35075,7 +35093,7 @@
         <v>2</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
@@ -35343,7 +35361,7 @@
         <v>3</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C43" s="19"/>
       <c r="D43" s="19"/>

</xml_diff>

<commit_message>
Remove bronchodilator I:E Ratio affect. Allow heart rate to change twice as fast in the new damper. Ventilator validation updates.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/CSTARS.xlsx
+++ b/data/human/adult/validation/Scenarios/CSTARS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFB3B9CB-DAC2-406C-AAAA-DD3A08BD3173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBC7FC2A-3718-4016-A032-676F46F87FDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28380" yWindow="1725" windowWidth="28875" windowHeight="28080" tabRatio="500" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25845" yWindow="2550" windowWidth="32595" windowHeight="26535" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Scenario1" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1355" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1337" uniqueCount="206">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -540,21 +540,10 @@
     <t>{ "SerializeState": { "Mode": "Save", "Filename": "CSTARS-Scenario2.json"} }</t>
   </si>
   <si>
-    <t xml:space="preserve">Learning Objectives:
- - Recognize worsening ARDS (moderate)
- - Adjust vent settings for safety
-Recommended Actions:
- - Increase FiO2 to 0.5
-</t>
-  </si>
-  <si>
     <t>VT (measured)</t>
   </si>
   <si>
     <t xml:space="preserve">A 22 year-old soldier was involved in a motor vehicle crash with rollover and ejection from the vehicle.  He suffered multiple rib fractures, a right femur fracture, multiple lacerations and pulmonary contusion.  He underwent internal fixation of the femur fracture, received 4 units of whole blood, had a chest tube placed for a small hemothorax and returned from the operating room on mechanical ventilation. The patient is sedated and is not currently triggering the ventilator.  Intraoperatively 3 L of crystalloids were administered. The patient is 6'2" tall, weighs 200 lbs and has no known comorbidities or allergies.  Chest radiograph demonstrates bi-basilar early consolidation, presence of the chest tube and pulmonary contusion. </t>
-  </si>
-  <si>
-    <t>A 62 year-old contractor developed pneumonia while working on a water purification system. He has 90- pack year history of cigarette smoking (2 packs per day x 45 years), has type II diabetes and primary hypertension managed with oral medications. He uses a rescue inhaler (albuterol) and is on a maintenance inhaled corticosteroid. His pre-deployment FEV-1 is 65% of predicted. The patient is 5'9" tall, weighs 210 lbs and has no known allergies. Chest radiograph demonstrates left-lower lobe consolidation, haziness in the right lower lobe, flattened diaphragms and hyperinflation in the upper lung fields. Heart rate is normal sinus rhythm and occasional PVC's. Patient is sedated and not triggering ventilator.</t>
   </si>
   <si>
     <t xml:space="preserve">    { "PatientAction": { "ChronicObstructivePulmonaryDiseaseExacerbation":
@@ -618,82 +607,11 @@
     <t>{ "SerializeState": { "Mode": "Save", "Filename": "CSTARS-Scenario4.json"} }</t>
   </si>
   <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 59, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>Patient transport continues.
-Learning Objectives:
- - Recognize need to increase PEEP to keep on PEEP matrix
-Recommended Actions:
- - Increase PEEP to 10 to keep on PEEP matrix
-Ventilator settings are updated to:
- - FiO2: 0.4 -&gt; 0.5
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.567    | NA          | 59          | NA  | 0.6    | 20      | 5            | 0.5 |</t>
-  </si>
-  <si>
-    <t>Patient transport continues.
-Learning Objectives:
- - Recognize improvement due to change in vent settings
- - Consider changing mode to address work shifting
-Recommended Actions:
- - Consider PC-CMV to liberate inspiratory volume and flow and reduce work shifting
- - Monitor for excessive tidal volume
-Ventilator settings are updated to:
- - PEEP: 5 -&gt; 10 cmH2O
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.567    | NA          | 59         | NA  | 0.6    | 20      | 10            | 0.5 |</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 59, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
     <t>Ventilator settings are (VT Target = 6.9 mL/kg (ideal)):
 &lt;br /&gt;
 | Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
 | VC-CMV | 0.567    | NA          | 59          | NA  | 0.6    | 20      | 5            | 0.4 |</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 59, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
   </si>
   <si>
     <t xml:space="preserve">    { "PatientAction": { "ChronicObstructivePulmonaryDiseaseExacerbation":
@@ -704,24 +622,6 @@
           { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.6 }}}]
       }}
     }</t>
-  </si>
-  <si>
-    <t>Learning Objectives:
- - Assess baseline status
-Recommended Actions:
- - Suspect dynamic airflow obstruction (high minute ventilation requirement but high SpO2 and low Pplat)
-&lt;br /&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Twenty minutes into the transport the patient is slightly agitated and is making inspiratory efforts that are not in sync with the ventilator.
-Learning Objectives:
- - Recognize increased airway resistance (PIP much higher than Pplat)
- - Recognize autoPEEP
- - Recognize failed trigger efforts due to autoPEEP (examine expiratory flow waveform)
-Recommended Actions:
- - Check airway patency (secretions?) suction ETT
- - Check breath sounds (wheezing?) - suspect bronchospasm and consider bronchodilator
-</t>
   </si>
   <si>
     <t>Patient suctioned and albuterol administered.
@@ -756,13 +656,6 @@
 &lt;br /&gt;</t>
   </si>
   <si>
-    <t>Learning Objectives:
- - Recognize mild ARDS
-Recommended Actions:
- - Increase RR to 23 to get acceptable pH
-&lt;br /&gt;</t>
-  </si>
-  <si>
     <t>{ "PatientAction": { "AcuteRespiratoryDistressSyndromeExacerbation":
   {
     "Severity": [ 
@@ -777,28 +670,6 @@
     "Severity": [ 
       { "Compartment": "LeftLung", "Severity": { "Scalar0To1": { "Value": 0.25 }}},
       { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.25 }}}]
-  }}
-}</t>
-  </si>
-  <si>
-    <t>Ventilator settings are (VT Target = 8.9 mL/kg (ideal)):
-&lt;br /&gt;
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.630    | NA          | 55          | NA  | 0.6    | 20       | 5            | 0.32 |</t>
-  </si>
-  <si>
-    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
-  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
-  "Mode": "AssistedControl", 
-  "InspirationWaveform": "Square",
-  "Flow": { "ScalarVolumePerTime": { "Value": 55, "Unit": "L/min" } },
-  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.32 } },
-  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
-  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
-  "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
-  "TidalVolume": { "ScalarVolume": { "Value": 630, "Unit": "mL" } },
-   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
   }}
 }</t>
   </si>
@@ -865,6 +736,53 @@
 | VC-CMV | 0.34   | NA          | 51           | NA  | 0.41  | 20       | 12            | 1.00 |</t>
   </si>
   <si>
+    <t>Ventilator settings are (VT Target = 6.9 mL/kg (ideal)):
+&lt;br /&gt;
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.488    | NA          | 52          | NA  | 0.6    | 20      | 5            | 0.4 |</t>
+  </si>
+  <si>
+    <t>Ventilator settings are (VT Target = 6.6 mL/kg (ideal)):
+&lt;br /&gt;
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.376    | NA          | 42          | NA  | 0.6    | 20      | 5            | 0.4 |</t>
+  </si>
+  <si>
+    <t>{ "PatientAction": { "PneumoniaExacerbation":
+  {
+    "Severity": [ 
+      { "Compartment": "LeftLung", "Severity": { "Scalar0To1": { "Value": 0.4 }}},
+      { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.4 }}}]
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "PatientAction": { "AcuteRespiratoryDistressSyndromeExacerbation":
+  {
+    "Severity": [ 
+      { "Compartment": "LeftLung", "Severity": { "Scalar0To1": { "Value": 0.91 }}},
+      { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.91 }}}]
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 59, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
     <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
   { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
   "Mode": "AssistedControl", 
@@ -875,16 +793,9 @@
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 12, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
   "TidalVolume": { "ScalarVolume": { "Value": 340, "Unit": "mL" } },
-   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
+   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
-  </si>
-  <si>
-    <t>Ventilator settings are (VT Target = 6.9 mL/kg (ideal)):
-&lt;br /&gt;
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.488    | NA          | 52          | NA  | 0.6    | 20      | 5            | 0.4 |</t>
   </si>
   <si>
     <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
@@ -897,16 +808,9 @@
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
   "TidalVolume": { "ScalarVolume": { "Value": 488, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
-  </si>
-  <si>
-    <t>Ventilator settings are (VT Target = 6.6 mL/kg (ideal)):
-&lt;br /&gt;
-| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
-| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| VC-CMV | 0.376    | NA          | 42          | NA  | 0.6    | 20      | 5            | 0.4 |</t>
   </si>
   <si>
     <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
@@ -919,25 +823,7 @@
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
   "TidalVolume": { "ScalarVolume": { "Value": 376, "Unit": "mL" } },
-  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "PatientAction": { "PneumoniaExacerbation":
-  {
-    "Severity": [ 
-      { "Compartment": "LeftLung", "Severity": { "Scalar0To1": { "Value": 0.4 }}},
-      { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.4 }}}]
-  }}
-}</t>
-  </si>
-  <si>
-    <t>{ "PatientAction": { "AcuteRespiratoryDistressSyndromeExacerbation":
-  {
-    "Severity": [ 
-      { "Compartment": "LeftLung", "Severity": { "Scalar0To1": { "Value": 0.91 }}},
-      { "Compartment": "RightLung", "Severity": { "Scalar0To1": { "Value": 0.91 }}}]
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
   </si>
@@ -948,10 +834,10 @@
   "InspirationWaveform": "Square",
   "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.6 } },
   "InspiratoryPeriod": { "ScalarTime": { "Value": 1.2, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 22, "Unit": "cmH2O" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 18.5, "Unit": "cmH2O" } },
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 8, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 10, "Unit": "1/min" } },
-   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
+   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
   </si>
@@ -961,7 +847,15 @@
 &lt;br /&gt;
 | Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| PC-CMV | NA     | 22          | NA           | NA  | 1.2    | 10       | 8            | 0.60 |</t>
+| PC-CMV | NA     | 18.5          | NA           | NA  | 1.2    | 10       | 8            | 0.60 |</t>
+  </si>
+  <si>
+    <t>&lt;br /&gt;
+Ventilator settings are (delivered VT of 460 ml):
+&lt;br /&gt;
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| PC-CMV | NA     | 15          | NA           | NA  | 1.3    | 10       | 5            | 0.40 |</t>
   </si>
   <si>
     <t>{ "EquipmentAction": { "MechanicalVentilatorPressureControl": { "MechanicalVentilatorMode": 
@@ -970,20 +864,131 @@
   "InspirationWaveform": "Square",
   "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
   "InspiratoryPeriod": { "ScalarTime": { "Value": 1.3, "Unit": "s" } },
-  "InspiratoryPressure": { "ScalarPressure": { "Value": 18, "Unit": "cmH2O" } },
+  "InspiratoryPressure": { "ScalarPressure": { "Value": 15, "Unit": "cmH2O" } },
   "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
   "RespirationRate": { "ScalarFrequency": { "Value": 10, "Unit": "1/min" } },
-   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -2.0, "Unit": "cmH2O"  } }
+   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
   }}
 }</t>
   </si>
   <si>
-    <t>&lt;br /&gt;
-Ventilator settings are (delivered VT of 460 ml):
+    <t>Learning Objectives:
+ - Recognize mild ARDS
+ - Recognize acceptable ventilator settings
+Recommended Actions:
+ - None
+&lt;br /&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learning Objectives:
+ - Recognize worsening ARDS (moderate)
+ - Adjust vent settings for safety
+Recommended Actions:
+ - Increase FiO2 to 0.5
+ - Decrease VT to 490 mL to get acceptable DP
+</t>
+  </si>
+  <si>
+    <t>A 62 year-old contractor developed pneumonia while working on a water purification system. He has 90- pack year history of cigarette smoking (2 packs per day x 45 years), has type II diabetes and primary hypertension managed with oral medications. He uses a rescue inhaler (albuterol) and is on a maintenance inhaled corticosteroid. His pre-deployment FEV-1 is 43% of predicted. The patient is 5'9" tall, weighs 210 lbs and has no known allergies. Chest radiograph demonstrates left-lower lobe consolidation, haziness in the right lower lobe, flattened diaphragms and hyperinflation in the upper lung fields. Heart rate is normal sinus rhythm and occasional PVC's. Patient is sedated and not triggering ventilator.</t>
+  </si>
+  <si>
+    <t>Learning Objectives:
+ - Assess baseline status
+ - Recognize presence of autoPEEP (from flow waveform)
+ - Suspect obstructive lung disease (high minute ventilation requirement but high SpO2 and low Pplat)
+Recommended Actions:
+ - None
+&lt;br /&gt;</t>
+  </si>
+  <si>
+    <t>Twenty minutes into the transport the patient is slightly agitated and is making inspiratory efforts that are not in sync with the ventilator.
+Learning Objectives:
+ - Recognize increased airway resistance (PIP much higher than Pplat)
+ - Recognize autoPEEP (from flow waveform)
+ - Recognize failed trigger efforts due to autoPEEP (examine expiratory flow waveform)
+Recommended Actions:
+ - Goal shifts to Comfort (improve synchrony) due to failed trigger efforts
+ - Check airway patency (secretions?) suction ETT
+ - Check breath sounds (wheezing?) - suspect bronchospasm and consider bronchodilator</t>
+  </si>
+  <si>
+    <t>Patient transport has ended. 
+Learning Objectives:
+ - Recognize improvement due to change in vent settings
+ - Consider changing mode to address work shifting
+Recommended Actions:
+ - None
+Ventilator settings are updated to:
+ - PEEP: 5 -&gt; 10 cmH2O
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.567    | NA          | 50         | NA  | 0.6    | 20      | 10            | 0.5 |</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 50, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 10, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 567, "Unit": "mL" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 50, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.5 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 20, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 490, "Unit": "mL" } },
+  "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
+  </si>
+  <si>
+    <t>Patient transport continues.
+Learning Objectives:
+ - Recognize need to increase PEEP to keep on PEEP matrix
+Recommended Actions:
+ - Increase PEEP to 10 to keep on PEEP matrix
+Ventilator settings are updated to:
+ - FiO2: 0.4 -&gt; 0.5
+ - VT: 567 -&gt; 490 mL
+ - Flow: 59 -&gt; 50 L/min
+| Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
+| ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
+| VC-CMV | 0.490    | NA          | 50          | NA  | 0.6    | 20      | 5            | 0.5 |</t>
+  </si>
+  <si>
+    <t>Ventilator settings are (VT Target = 8.9 mL/kg (ideal)):
 &lt;br /&gt;
 | Mode   | VT (L) | PIP (cmH2O) | Flow (L/min) | I:E | TI (s) | RR (bpm) | PEEP (cmH2O) | FiO2 |
 | ------ | ------ | ----------- | ------------ | --- | ------ | -------- | ------------ | ---- |
-| PC-CMV | NA     | 18          | NA           | NA  | 1.3    | 10       | 5            | 0.40 |</t>
+| VC-CMV | 0.630    | NA          | 55          | NA  | 0.6    | 18       | 5            | 0.4 |</t>
+  </si>
+  <si>
+    <t>{ "EquipmentAction": { "MechanicalVentilatorVolumeControl": { "MechanicalVentilatorMode": 
+  { "MechanicalVentilatorAction": { "EquipmentAction": { "Action": {} } }, "Connection": "On" },
+  "Mode": "AssistedControl", 
+  "InspirationWaveform": "Square",
+  "Flow": { "ScalarVolumePerTime": { "Value": 55, "Unit": "L/min" } },
+  "FractionInspiredOxygen": { "Scalar0To1": { "Value": 0.4 } },
+  "InspiratoryPeriod": { "ScalarTime": { "Value": 0.6, "Unit": "s" } },
+  "PositiveEndExpiratoryPressure": { "ScalarPressure": { "Value": 5, "Unit": "cmH2O" } },
+  "RespirationRate": { "ScalarFrequency": { "Value": 18, "Unit": "1/min" } },
+  "TidalVolume": { "ScalarVolume": { "Value": 630, "Unit": "mL" } },
+   "InspirationPatientTriggerPressure": { "ScalarPressure": { "Value": -1.0, "Unit": "cmH2O"  } }
+  }}
+}</t>
   </si>
 </sst>
 </file>
@@ -1221,6 +1226,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1229,9 +1237,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1642,7 +1647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ57"/>
+  <dimension ref="A1:AMJ54"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="12" customWidth="1"/>
@@ -1692,7 +1697,7 @@
         <v>81</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G2" s="25"/>
       <c r="H2" s="25"/>
@@ -1723,11 +1728,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>9</v>
@@ -1805,13 +1810,13 @@
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>7</v>
       </c>
@@ -1823,13 +1828,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>23</v>
@@ -1839,15 +1844,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>181</v>
-      </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="B12" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -1855,13 +1860,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>25</v>
@@ -1871,13 +1876,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1885,15 +1890,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
+      <c r="B15" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="21"/>
       <c r="G15" s="9" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -1901,13 +1906,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -1957,7 +1962,7 @@
         <v>113</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H18" s="10"/>
     </row>
@@ -2109,13 +2114,13 @@
       <c r="A25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
       <c r="G25" s="1" t="s">
         <v>7</v>
       </c>
@@ -2127,13 +2132,13 @@
       <c r="A26" s="8">
         <v>2</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="19" t="s">
         <v>141</v>
       </c>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
     </row>
@@ -2141,13 +2146,13 @@
       <c r="A27" s="8">
         <v>2</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
       <c r="G27" s="9" t="s">
         <v>110</v>
       </c>
@@ -2157,15 +2162,15 @@
       <c r="A28" s="8">
         <v>2</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
       <c r="G28" s="9" t="s">
-        <v>143</v>
+        <v>196</v>
       </c>
       <c r="H28" s="9"/>
     </row>
@@ -2173,13 +2178,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
       <c r="G29" s="9"/>
       <c r="H29" s="9"/>
     </row>
@@ -2229,7 +2234,7 @@
         <v>113</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H31" s="10"/>
     </row>
@@ -2377,235 +2382,219 @@
       </c>
       <c r="H37" s="10"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38" s="2" t="s">
+    <row r="38" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B38" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H38" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="263.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="8">
+        <v>3</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>202</v>
+      </c>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="H39" s="10"/>
+    </row>
+    <row r="40" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="8">
+        <v>3</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="10"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A41" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H41" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D38" s="2" t="s">
+      <c r="B42" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E42" s="2">
+        <v>490</v>
+      </c>
+      <c r="F42" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="H42" s="10"/>
+    </row>
+    <row r="43" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E38" s="2">
-        <v>1</v>
-      </c>
-      <c r="F38" s="11" t="s">
+      <c r="E43" s="2">
+        <v>2</v>
+      </c>
+      <c r="F43" s="11" t="s">
         <v>107</v>
       </c>
-      <c r="G38" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="H38" s="10"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E39" s="2">
-        <v>1</v>
-      </c>
-      <c r="F39" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="G39" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="H39" s="10"/>
-    </row>
-    <row r="40" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B40" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="C40" s="21"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
-      <c r="G40" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H40" s="15" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="225.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="8">
-        <v>3</v>
-      </c>
-      <c r="B41" s="18" t="s">
-        <v>170</v>
-      </c>
-      <c r="C41" s="19"/>
-      <c r="D41" s="19"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="H41" s="10"/>
-    </row>
-    <row r="42" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="8">
-        <v>3</v>
-      </c>
-      <c r="B42" s="18" t="s">
-        <v>112</v>
-      </c>
-      <c r="C42" s="18"/>
-      <c r="D42" s="18"/>
-      <c r="E42" s="18"/>
-      <c r="F42" s="18"/>
-      <c r="G42" s="9"/>
-      <c r="H42" s="10"/>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A43" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G43" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H43" s="15" t="s">
-        <v>8</v>
-      </c>
+      <c r="G43" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H43" s="10"/>
     </row>
     <row r="44" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>64</v>
+        <v>116</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>32</v>
+        <v>135</v>
       </c>
       <c r="E44" s="2">
-        <v>567</v>
+        <v>2</v>
       </c>
       <c r="F44" s="11" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="H44" s="10"/>
     </row>
-    <row r="45" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E45" s="2">
-        <v>2</v>
-      </c>
-      <c r="F45" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="H45" s="10"/>
-    </row>
-    <row r="46" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C46" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E46" s="2">
-        <v>2</v>
-      </c>
-      <c r="F46" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>80</v>
+    <row r="45" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B45" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H45" s="15" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="260.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="8">
+        <v>4</v>
+      </c>
+      <c r="B46" s="19" t="s">
+        <v>201</v>
+      </c>
+      <c r="C46" s="20"/>
+      <c r="D46" s="20"/>
+      <c r="E46" s="20"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="9" t="s">
+        <v>200</v>
       </c>
       <c r="H46" s="10"/>
     </row>
-    <row r="47" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="E47" s="2">
-        <v>2</v>
-      </c>
-      <c r="F47" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="G47" s="2" t="s">
-        <v>117</v>
-      </c>
+    <row r="47" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="8">
+        <v>4</v>
+      </c>
+      <c r="B47" s="19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C47" s="19"/>
+      <c r="D47" s="19"/>
+      <c r="E47" s="19"/>
+      <c r="F47" s="19"/>
+      <c r="G47" s="9"/>
       <c r="H47" s="10"/>
     </row>
-    <row r="48" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B48" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="C48" s="21"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A48" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>29</v>
+      </c>
       <c r="G48" s="1" t="s">
         <v>7</v>
       </c>
@@ -2613,83 +2602,99 @@
         <v>8</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="260.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="8">
-        <v>4</v>
-      </c>
-      <c r="B49" s="18" t="s">
-        <v>165</v>
-      </c>
-      <c r="C49" s="19"/>
-      <c r="D49" s="19"/>
-      <c r="E49" s="19"/>
-      <c r="F49" s="20"/>
-      <c r="G49" s="9" t="s">
-        <v>167</v>
+    <row r="49" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E49" s="2">
+        <v>490</v>
+      </c>
+      <c r="F49" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>143</v>
       </c>
       <c r="H49" s="10"/>
     </row>
-    <row r="50" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="8">
-        <v>4</v>
-      </c>
-      <c r="B50" s="18" t="s">
-        <v>112</v>
-      </c>
-      <c r="C50" s="18"/>
-      <c r="D50" s="18"/>
-      <c r="E50" s="18"/>
-      <c r="F50" s="18"/>
-      <c r="G50" s="9"/>
+    <row r="50" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="E50" s="2">
+        <v>3</v>
+      </c>
+      <c r="F50" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="G50" s="13" t="s">
+        <v>76</v>
+      </c>
       <c r="H50" s="10"/>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A51" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H51" s="15" t="s">
-        <v>8</v>
-      </c>
+    <row r="51" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E51" s="2">
+        <v>3</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="H51" s="10"/>
     </row>
     <row r="52" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>64</v>
+        <v>37</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="E52" s="2">
-        <v>567</v>
+        <v>3</v>
       </c>
       <c r="F52" s="11" t="s">
         <v>134</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>144</v>
+        <v>80</v>
       </c>
       <c r="H52" s="10"/>
     </row>
@@ -2698,10 +2703,10 @@
         <v>30</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D53" s="2" t="s">
         <v>47</v>
@@ -2710,114 +2715,58 @@
         <v>3</v>
       </c>
       <c r="F53" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="G53" s="13" t="s">
-        <v>76</v>
+        <v>134</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>119</v>
       </c>
       <c r="H53" s="10"/>
     </row>
     <row r="54" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>35</v>
+        <v>116</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>135</v>
+        <v>49</v>
       </c>
       <c r="E54" s="2">
         <v>3</v>
       </c>
       <c r="F54" s="11" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>79</v>
+        <v>117</v>
       </c>
       <c r="H54" s="10"/>
-    </row>
-    <row r="55" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E55" s="2">
-        <v>3</v>
-      </c>
-      <c r="F55" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="G55" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="H55" s="10"/>
-    </row>
-    <row r="56" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E56" s="2">
-        <v>3</v>
-      </c>
-      <c r="F56" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="G56" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="H56" s="10"/>
-    </row>
-    <row r="57" spans="1:8" s="12" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E57" s="2">
-        <v>3</v>
-      </c>
-      <c r="F57" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="G57" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H57" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="B48:F48"/>
-    <mergeCell ref="B49:F49"/>
-    <mergeCell ref="B50:F50"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B39:F39"/>
+    <mergeCell ref="B40:F40"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B38:F38"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B45:F45"/>
+    <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B47:F47"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="F1:H1"/>
@@ -2831,22 +2780,6 @@
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B41:F41"/>
-    <mergeCell ref="B42:F42"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B40:F40"/>
-    <mergeCell ref="B27:F27"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -2865,9 +2798,9 @@
     <col min="1" max="1" width="24.85546875" style="12" customWidth="1"/>
     <col min="2" max="2" width="36.28515625" style="12" customWidth="1"/>
     <col min="3" max="3" width="15" style="12" customWidth="1"/>
-    <col min="4" max="4" width="25" style="12" customWidth="1"/>
-    <col min="5" max="5" width="35.5703125" style="12" customWidth="1"/>
-    <col min="6" max="6" width="41.85546875" style="12" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.42578125" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="38.5703125" style="12" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="83.85546875" style="12" customWidth="1"/>
     <col min="8" max="8" width="33.85546875" style="16" customWidth="1"/>
     <col min="9" max="1024" width="11.5703125" style="12"/>
@@ -2907,7 +2840,7 @@
         <v>82</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>146</v>
+        <v>197</v>
       </c>
       <c r="G2" s="25"/>
       <c r="H2" s="25"/>
@@ -2936,11 +2869,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>9</v>
@@ -3024,13 +2957,13 @@
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>7</v>
       </c>
@@ -3042,31 +2975,31 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:1024" ht="154.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:1024" ht="179.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>147</v>
-      </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="B12" s="19" t="s">
+        <v>145</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
-        <v>172</v>
+        <v>198</v>
       </c>
       <c r="H12" s="10"/>
     </row>
@@ -3074,13 +3007,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="10"/>
     </row>
@@ -3088,13 +3021,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="10"/>
     </row>
@@ -3102,15 +3035,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>183</v>
-      </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
+      <c r="B15" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>182</v>
+        <v>204</v>
       </c>
       <c r="H15" s="10"/>
     </row>
@@ -3118,13 +3051,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="10"/>
     </row>
@@ -3174,7 +3107,7 @@
         <v>113</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H18" s="10"/>
     </row>
@@ -3198,7 +3131,7 @@
         <v>137</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="H19" s="10"/>
     </row>
@@ -3222,7 +3155,7 @@
         <v>138</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H20" s="10"/>
     </row>
@@ -3246,7 +3179,7 @@
         <v>114</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="H21" s="10"/>
     </row>
@@ -3270,7 +3203,7 @@
         <v>139</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="H22" s="10"/>
     </row>
@@ -3294,7 +3227,7 @@
         <v>140</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="H23" s="10"/>
     </row>
@@ -3302,13 +3235,13 @@
       <c r="A24" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
       <c r="G24" s="1" t="s">
         <v>7</v>
       </c>
@@ -3320,13 +3253,13 @@
       <c r="A25" s="8">
         <v>2</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="19" t="s">
         <v>142</v>
       </c>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
     </row>
@@ -3334,15 +3267,15 @@
       <c r="A26" s="8">
         <v>2</v>
       </c>
-      <c r="B26" s="18" t="s">
-        <v>171</v>
-      </c>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="B26" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="9" t="s">
-        <v>173</v>
+        <v>199</v>
       </c>
       <c r="H26" s="9"/>
     </row>
@@ -3364,13 +3297,13 @@
       <c r="A28" s="8">
         <v>2</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
       <c r="G28" s="9"/>
       <c r="H28" s="10"/>
     </row>
@@ -3420,7 +3353,7 @@
         <v>113</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H30" s="10"/>
     </row>
@@ -3524,13 +3457,13 @@
       <c r="A35" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
       <c r="G35" s="1" t="s">
         <v>7</v>
       </c>
@@ -3542,15 +3475,15 @@
       <c r="A36" s="8">
         <v>3</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="19"/>
       <c r="G36" s="9" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="H36" s="10"/>
     </row>
@@ -3558,13 +3491,13 @@
       <c r="A37" s="8">
         <v>3</v>
       </c>
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="18"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="19"/>
+      <c r="F37" s="19"/>
       <c r="G37" s="9"/>
       <c r="H37" s="10"/>
     </row>
@@ -3614,7 +3547,7 @@
         <v>113</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H39" s="10"/>
     </row>
@@ -3716,26 +3649,6 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="B24:F24"/>
     <mergeCell ref="B36:F36"/>
@@ -3745,6 +3658,26 @@
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -3803,7 +3736,7 @@
         <v>83</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="G2" s="25"/>
       <c r="H2" s="25"/>
@@ -3830,11 +3763,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>9</v>
@@ -3918,13 +3851,13 @@
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>7</v>
       </c>
@@ -3939,10 +3872,10 @@
       <c r="B11" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="21"/>
       <c r="G11" s="9"/>
       <c r="H11" s="10" t="s">
         <v>23</v>
@@ -3952,15 +3885,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>180</v>
-      </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="B12" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="H12" s="10"/>
     </row>
@@ -3968,13 +3901,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="10" t="s">
         <v>25</v>
@@ -3984,13 +3917,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="10"/>
     </row>
@@ -3998,15 +3931,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>193</v>
-      </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
+      <c r="B15" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="H15" s="10"/>
     </row>
@@ -4014,13 +3947,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="10"/>
     </row>
@@ -4070,7 +4003,7 @@
         <v>113</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H18" s="10"/>
     </row>
@@ -4222,13 +4155,13 @@
       <c r="A25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
       <c r="G25" s="1" t="s">
         <v>7</v>
       </c>
@@ -5256,13 +5189,13 @@
       <c r="A26" s="8">
         <v>2</v>
       </c>
-      <c r="B26" s="18" t="s">
-        <v>160</v>
-      </c>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="B26" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
     </row>
@@ -5270,15 +5203,15 @@
       <c r="A27" s="8">
         <v>2</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
       <c r="G27" s="9" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="H27" s="10"/>
       <c r="I27" s="14"/>
@@ -6302,15 +6235,15 @@
       <c r="A28" s="8">
         <v>2</v>
       </c>
-      <c r="B28" s="18" t="s">
-        <v>201</v>
-      </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="B28" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
       <c r="G28" s="9" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="H28" s="10"/>
       <c r="I28" s="14"/>
@@ -7334,13 +7267,13 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="19"/>
+      <c r="F29" s="19"/>
       <c r="H29" s="10"/>
       <c r="I29" s="14"/>
       <c r="J29" s="14"/>
@@ -9421,7 +9354,7 @@
         <v>113</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H31" s="10"/>
     </row>
@@ -9445,7 +9378,7 @@
         <v>113</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="H32" s="10"/>
     </row>
@@ -9469,7 +9402,7 @@
         <v>113</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H33" s="10"/>
     </row>
@@ -9493,7 +9426,7 @@
         <v>114</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H34" s="10"/>
     </row>
@@ -9517,7 +9450,7 @@
         <v>114</v>
       </c>
       <c r="G35" s="13" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="H35" s="10"/>
     </row>
@@ -9541,7 +9474,7 @@
         <v>114</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="H36" s="10"/>
     </row>
@@ -9556,7 +9489,7 @@
         <v>36</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E37" s="2">
         <v>100</v>
@@ -9565,7 +9498,7 @@
         <v>121</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="H37" s="10"/>
     </row>
@@ -9573,13 +9506,13 @@
       <c r="A38" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="B38" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="21"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="21"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
       <c r="G38" s="1" t="s">
         <v>7</v>
       </c>
@@ -10607,15 +10540,15 @@
       <c r="A39" s="8">
         <v>3</v>
       </c>
-      <c r="B39" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
+      <c r="B39" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
       <c r="G39" s="9" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="H39" s="10"/>
       <c r="I39" s="14"/>
@@ -11639,13 +11572,13 @@
       <c r="A40" s="8">
         <v>3</v>
       </c>
-      <c r="B40" s="18" t="s">
+      <c r="B40" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="18"/>
+      <c r="C40" s="19"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="19"/>
+      <c r="F40" s="19"/>
       <c r="G40" s="9"/>
       <c r="H40" s="10"/>
       <c r="I40" s="14"/>
@@ -13727,7 +13660,7 @@
         <v>113</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H42" s="10"/>
     </row>
@@ -13757,25 +13690,6 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B29:F29"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="B39:F39"/>
@@ -13786,6 +13700,25 @@
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -13871,11 +13804,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>9</v>
@@ -13959,13 +13892,13 @@
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>7</v>
       </c>
@@ -13977,13 +13910,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="10" t="s">
         <v>23</v>
@@ -13993,13 +13926,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>90</v>
       </c>
@@ -14009,13 +13942,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9"/>
       <c r="H13" s="10" t="s">
         <v>25</v>
@@ -14025,13 +13958,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="10"/>
     </row>
@@ -14039,15 +13972,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>197</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
+      <c r="B15" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="21"/>
       <c r="G15" s="9" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
       <c r="H15" s="10"/>
     </row>
@@ -14055,13 +13988,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9"/>
       <c r="H16" s="10"/>
     </row>
@@ -14111,7 +14044,7 @@
         <v>113</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H18" s="10"/>
     </row>
@@ -14263,13 +14196,13 @@
       <c r="A25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
       <c r="G25" s="1" t="s">
         <v>7</v>
       </c>
@@ -14281,13 +14214,13 @@
       <c r="A26" s="8">
         <v>2</v>
       </c>
-      <c r="B26" s="18" t="s">
-        <v>164</v>
-      </c>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="B26" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
     </row>
@@ -14295,13 +14228,13 @@
       <c r="A27" s="8">
         <v>2</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
       <c r="G27" s="9" t="s">
         <v>91</v>
       </c>
@@ -14311,15 +14244,15 @@
       <c r="A28" s="8">
         <v>2</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
       <c r="G28" s="9" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="H28" s="10"/>
     </row>
@@ -14369,7 +14302,7 @@
         <v>113</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H30" s="10"/>
     </row>
@@ -14521,13 +14454,13 @@
       <c r="A37" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B37" s="21" t="s">
+      <c r="B37" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="21"/>
-      <c r="D37" s="21"/>
-      <c r="E37" s="21"/>
-      <c r="F37" s="21"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
       <c r="G37" s="1" t="s">
         <v>7</v>
       </c>
@@ -14539,13 +14472,13 @@
       <c r="A38" s="8">
         <v>3</v>
       </c>
-      <c r="B38" s="18" t="s">
+      <c r="B38" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
+      <c r="C38" s="19"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="19"/>
+      <c r="F38" s="19"/>
       <c r="G38" s="9" t="s">
         <v>92</v>
       </c>
@@ -14555,13 +14488,13 @@
       <c r="A39" s="8">
         <v>3</v>
       </c>
-      <c r="B39" s="18" t="s">
+      <c r="B39" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
+      <c r="C39" s="19"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="19"/>
+      <c r="F39" s="19"/>
       <c r="G39" s="9"/>
       <c r="H39" s="10"/>
     </row>
@@ -14611,7 +14544,7 @@
         <v>113</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H41" s="10"/>
     </row>
@@ -14761,25 +14694,6 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B37:F37"/>
     <mergeCell ref="B38:F38"/>
     <mergeCell ref="B39:F39"/>
@@ -14789,6 +14703,25 @@
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -14874,11 +14807,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>9</v>
@@ -14962,13 +14895,13 @@
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>7</v>
       </c>
@@ -14980,13 +14913,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="10" t="s">
         <v>23</v>
@@ -14996,13 +14929,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>99</v>
       </c>
@@ -15012,13 +14945,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9" t="s">
         <v>93</v>
       </c>
@@ -15030,13 +14963,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9"/>
       <c r="H14" s="10"/>
     </row>
@@ -15044,15 +14977,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="20"/>
+      <c r="B15" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="21"/>
       <c r="G15" s="9" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="H15" s="10"/>
     </row>
@@ -15060,15 +14993,15 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B16" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="19"/>
       <c r="G16" s="9" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="H16" s="10"/>
     </row>
@@ -15118,7 +15051,7 @@
         <v>113</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H18" s="10"/>
     </row>
@@ -15270,13 +15203,13 @@
       <c r="A25" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
       <c r="G25" s="1" t="s">
         <v>7</v>
       </c>
@@ -15288,13 +15221,13 @@
       <c r="A26" s="8">
         <v>2</v>
       </c>
-      <c r="B26" s="18" t="s">
-        <v>163</v>
-      </c>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="B26" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="9"/>
       <c r="H26" s="9"/>
     </row>
@@ -15302,13 +15235,13 @@
       <c r="A27" s="8">
         <v>2</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
       <c r="G27" s="9" t="s">
         <v>94</v>
       </c>
@@ -15318,15 +15251,15 @@
       <c r="A28" s="8">
         <v>2</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
       <c r="G28" s="9" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="H28" s="10"/>
     </row>
@@ -15376,7 +15309,7 @@
         <v>113</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H30" s="10"/>
     </row>
@@ -15480,13 +15413,13 @@
       <c r="A35" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C35" s="21"/>
-      <c r="D35" s="21"/>
-      <c r="E35" s="21"/>
-      <c r="F35" s="21"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
       <c r="G35" s="1" t="s">
         <v>7</v>
       </c>
@@ -15498,13 +15431,13 @@
       <c r="A36" s="8">
         <v>3</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="19"/>
       <c r="G36" s="9" t="s">
         <v>95</v>
       </c>
@@ -15514,13 +15447,13 @@
       <c r="A37" s="8">
         <v>3</v>
       </c>
-      <c r="B37" s="18" t="s">
+      <c r="B37" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="18"/>
+      <c r="C37" s="19"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="19"/>
+      <c r="F37" s="19"/>
       <c r="G37" s="9"/>
       <c r="H37" s="10"/>
     </row>
@@ -15570,7 +15503,7 @@
         <v>113</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H39" s="10"/>
     </row>
@@ -15672,25 +15605,6 @@
     </row>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="E5:F9"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B35:F35"/>
     <mergeCell ref="B36:F36"/>
     <mergeCell ref="B37:F37"/>
@@ -15700,6 +15614,25 @@
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="B28:F28"/>
     <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="E5:F9"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -15785,11 +15718,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>9</v>
@@ -15873,13 +15806,13 @@
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>7</v>
       </c>
@@ -15891,13 +15824,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="10" t="s">
         <v>23</v>
@@ -15907,15 +15840,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>200</v>
-      </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="B12" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="H12" s="10"/>
     </row>
@@ -15923,13 +15856,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9" t="s">
         <v>63</v>
       </c>
@@ -15940,14 +15873,14 @@
         <v>1</v>
       </c>
       <c r="B14" s="30" t="s">
-        <v>202</v>
-      </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="20"/>
+        <v>191</v>
+      </c>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="21"/>
       <c r="G14" s="9" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="H14" s="10"/>
     </row>
@@ -15955,15 +15888,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="H15" s="10"/>
     </row>
@@ -16013,7 +15946,7 @@
         <v>113</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H17" s="10"/>
     </row>
@@ -16165,13 +16098,13 @@
       <c r="A24" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
       <c r="G24" s="1" t="s">
         <v>7</v>
       </c>
@@ -16183,13 +16116,13 @@
       <c r="A25" s="8">
         <v>2</v>
       </c>
-      <c r="B25" s="18" t="s">
-        <v>162</v>
-      </c>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
+      <c r="B25" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
     </row>
@@ -16197,13 +16130,13 @@
       <c r="A26" s="8">
         <v>2</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="9" t="s">
         <v>100</v>
       </c>
@@ -16213,15 +16146,15 @@
       <c r="A27" s="8">
         <v>2</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
       <c r="G27" s="9" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="H27" s="10"/>
     </row>
@@ -16271,7 +16204,7 @@
         <v>113</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H29" s="10"/>
     </row>
@@ -16375,13 +16308,13 @@
       <c r="A34" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
       <c r="G34" s="1" t="s">
         <v>7</v>
       </c>
@@ -16393,13 +16326,13 @@
       <c r="A35" s="8">
         <v>3</v>
       </c>
-      <c r="B35" s="18" t="s">
+      <c r="B35" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
       <c r="G35" s="9" t="s">
         <v>96</v>
       </c>
@@ -16409,13 +16342,13 @@
       <c r="A36" s="8">
         <v>3</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="19"/>
       <c r="G36" s="9"/>
       <c r="H36" s="10"/>
     </row>
@@ -16459,13 +16392,13 @@
         <v>32</v>
       </c>
       <c r="E38" s="2">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="F38" s="11" t="s">
         <v>113</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H38" s="10"/>
     </row>
@@ -16567,12 +16500,19 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -16581,19 +16521,12 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -16679,11 +16612,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>9</v>
@@ -16767,13 +16700,13 @@
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
       <c r="G10" s="1" t="s">
         <v>7</v>
       </c>
@@ -16785,13 +16718,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
       <c r="G11" s="9"/>
       <c r="H11" s="10" t="s">
         <v>23</v>
@@ -16801,13 +16734,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>108</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
       <c r="G12" s="9" t="s">
         <v>98</v>
       </c>
@@ -16817,13 +16750,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="B13" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="9" t="s">
         <v>63</v>
       </c>
@@ -16833,15 +16766,15 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="B14" s="19" t="s">
+        <v>194</v>
+      </c>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
       <c r="G14" s="9" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
       <c r="H14" s="10"/>
     </row>
@@ -16849,15 +16782,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="B15" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
       <c r="G15" s="9" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="H15" s="10"/>
     </row>
@@ -16907,7 +16840,7 @@
         <v>113</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H17" s="10"/>
     </row>
@@ -17059,13 +16992,13 @@
       <c r="A24" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="21"/>
-      <c r="D24" s="21"/>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
       <c r="G24" s="1" t="s">
         <v>7</v>
       </c>
@@ -17077,13 +17010,13 @@
       <c r="A25" s="8">
         <v>2</v>
       </c>
-      <c r="B25" s="18" t="s">
-        <v>161</v>
-      </c>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
+      <c r="B25" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
     </row>
@@ -17091,13 +17024,13 @@
       <c r="A26" s="8">
         <v>2</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="19"/>
+      <c r="F26" s="19"/>
       <c r="G26" s="9" t="s">
         <v>101</v>
       </c>
@@ -17107,15 +17040,15 @@
       <c r="A27" s="8">
         <v>2</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C27" s="18"/>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="19"/>
+      <c r="F27" s="19"/>
       <c r="G27" s="9" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="H27" s="10"/>
     </row>
@@ -17165,7 +17098,7 @@
         <v>113</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H29" s="10"/>
     </row>
@@ -17269,13 +17202,13 @@
       <c r="A34" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="21"/>
-      <c r="D34" s="21"/>
-      <c r="E34" s="21"/>
-      <c r="F34" s="21"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
       <c r="G34" s="1" t="s">
         <v>7</v>
       </c>
@@ -17287,13 +17220,13 @@
       <c r="A35" s="8">
         <v>3</v>
       </c>
-      <c r="B35" s="18" t="s">
+      <c r="B35" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
       <c r="G35" s="9" t="s">
         <v>97</v>
       </c>
@@ -17303,13 +17236,13 @@
       <c r="A36" s="8">
         <v>3</v>
       </c>
-      <c r="B36" s="18" t="s">
+      <c r="B36" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
+      <c r="C36" s="19"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="19"/>
+      <c r="F36" s="19"/>
       <c r="G36" s="9"/>
       <c r="H36" s="10"/>
     </row>
@@ -17359,7 +17292,7 @@
         <v>113</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H38" s="10"/>
     </row>
@@ -17461,12 +17394,19 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:D2"/>
-    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="B35:F35"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="E5:F9"/>
@@ -17475,19 +17415,12 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="G9:H9"/>
     <mergeCell ref="G8:H8"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="B34:F34"/>
-    <mergeCell ref="B35:F35"/>
-    <mergeCell ref="B36:F36"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>